<commit_message>
Implementando auditoria de Difal por UF e FCP
</commit_message>
<xml_diff>
--- a/aliquotas.xlsx
+++ b/aliquotas.xlsx
@@ -8,17 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Faturamento\Desktop\nfe_sistema\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BAFB09B-D8EC-420E-B924-E917B43C5520}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E137CBC-D307-4AA1-8D3F-964228905309}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2304" windowWidth="23136" windowHeight="8880" xr2:uid="{9ADDC600-9F42-43BA-851C-A42DE1550295}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9ADDC600-9F42-43BA-851C-A42DE1550295}"/>
   </bookViews>
   <sheets>
-    <sheet name="ICMS" sheetId="1" r:id="rId1"/>
+    <sheet name="ICMS_DIFAL" sheetId="1" r:id="rId1"/>
     <sheet name="FCP" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">FCP!$A$1:$H$28</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">FCP!$A:$I</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">FCP!#REF!</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">FCP!#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="33">
   <si>
     <t>AC</t>
   </si>
@@ -125,179 +125,17 @@
     <t xml:space="preserve">RJ </t>
   </si>
   <si>
-    <t>Em destaque as alterações já realizadas em versões anteriores da tabela</t>
-  </si>
-  <si>
-    <t>Em destaque as alterações com relação à versão anterior da tabela</t>
-  </si>
-  <si>
-    <t>OBS.:</t>
-  </si>
-  <si>
-    <t>Alíquota única de 2.00</t>
-  </si>
-  <si>
-    <t>Fixo:2.00</t>
-  </si>
-  <si>
-    <t>TOCANTINS</t>
-  </si>
-  <si>
-    <t>UF com 2 alíquotas</t>
-  </si>
-  <si>
-    <t>Fixo:1.00</t>
-  </si>
-  <si>
-    <t>SERGIPE</t>
-  </si>
-  <si>
-    <t>SAO PAULO</t>
-  </si>
-  <si>
-    <t>UF não possi FCP e nem para comercialização</t>
-  </si>
-  <si>
-    <t>Fixo:0.00</t>
-  </si>
-  <si>
-    <t>SANTA CATARINA</t>
-  </si>
-  <si>
-    <t>Alíquota máxima de 2.00 (default)</t>
-  </si>
-  <si>
-    <t>Max:2.00</t>
-  </si>
-  <si>
-    <t>RORAIMA</t>
-  </si>
-  <si>
-    <t>RONDONIA</t>
-  </si>
-  <si>
-    <t>RIO GRANDE DO SUL</t>
-  </si>
-  <si>
-    <t>RIO GRANDE DO NORTE</t>
-  </si>
-  <si>
-    <t>UF com alíquota máxima de 4.00</t>
-  </si>
-  <si>
-    <t>Max:4.00</t>
-  </si>
-  <si>
-    <t>RIO DE JANEIRO</t>
-  </si>
-  <si>
-    <t>PIAUI</t>
-  </si>
-  <si>
-    <t>PERNAMBUCO</t>
-  </si>
-  <si>
-    <t>PARANA</t>
-  </si>
-  <si>
-    <t>PARAIBA</t>
-  </si>
-  <si>
-    <t>UF não possi FCP</t>
-  </si>
-  <si>
-    <t>PARA</t>
-  </si>
-  <si>
-    <t>Alíquota única de 2.00 a  partir de 01/01/24</t>
-  </si>
-  <si>
-    <t>Fixo: 2.00</t>
-  </si>
-  <si>
-    <t>MINAS GERAIS</t>
-  </si>
-  <si>
-    <t>MATO GROSSO DO SUL</t>
-  </si>
-  <si>
-    <t>MATO GROSSO</t>
-  </si>
-  <si>
-    <t>MARANHÃO</t>
-  </si>
-  <si>
-    <t>GOIAS</t>
-  </si>
-  <si>
-    <t>ESPIRITO SANTO</t>
-  </si>
-  <si>
-    <t>DISTRITO FEDERAL</t>
-  </si>
-  <si>
-    <t>Alíquota única de 2.00 a  partir de 01/02/24</t>
-  </si>
-  <si>
-    <t>CEARA</t>
-  </si>
-  <si>
-    <t>BAHIA</t>
-  </si>
-  <si>
-    <t>UF com até 2 Alíquotas possíveis (2025)</t>
-  </si>
-  <si>
-    <t>Fixo:1.20</t>
-  </si>
-  <si>
-    <t>AMAZONAS</t>
-  </si>
-  <si>
-    <t>AMAPA</t>
-  </si>
-  <si>
-    <t>UF com até 3 Alíquotas possíveis</t>
-  </si>
-  <si>
-    <t>ALAGOAS</t>
-  </si>
-  <si>
-    <t>UF não possui FCP</t>
-  </si>
-  <si>
-    <t>ACRE</t>
-  </si>
-  <si>
-    <t>Observação</t>
-  </si>
-  <si>
-    <t>.</t>
-  </si>
-  <si>
-    <t>Aliq_3</t>
-  </si>
-  <si>
-    <t>Aliq_2</t>
-  </si>
-  <si>
-    <t>Aliq_1</t>
-  </si>
-  <si>
-    <t>Nome UF</t>
-  </si>
-  <si>
     <t>UF</t>
   </si>
   <si>
-    <t>cUF</t>
+    <t>FCP</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -321,17 +159,8 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <u/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="8">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -350,32 +179,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF92D050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="13">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -503,69 +308,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -609,53 +356,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3400,619 +3102,238 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{219E7EC0-905D-4A02-91FD-4CCABD91BD06}">
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7" customWidth="1"/>
-    <col min="2" max="2" width="7" style="14" customWidth="1"/>
-    <col min="3" max="3" width="22" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="2" customWidth="1"/>
-    <col min="8" max="8" width="40.5546875" customWidth="1"/>
-    <col min="9" max="9" width="2.33203125" customWidth="1"/>
+    <col min="1" max="1" width="3.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.109375" style="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="33" t="s">
-        <v>86</v>
-      </c>
-      <c r="B1" s="32" t="s">
-        <v>85</v>
-      </c>
-      <c r="C1" s="31" t="s">
-        <v>84</v>
-      </c>
-      <c r="D1" s="31" t="s">
-        <v>83</v>
-      </c>
-      <c r="E1" s="31" t="s">
-        <v>82</v>
-      </c>
-      <c r="F1" s="31" t="s">
-        <v>81</v>
-      </c>
-      <c r="G1" s="31" t="s">
-        <v>80</v>
-      </c>
-      <c r="H1" s="30" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="28">
-        <v>12</v>
-      </c>
-      <c r="B2" s="29" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="27" t="s">
-        <v>78</v>
-      </c>
-      <c r="D2" s="28" t="s">
-        <v>42</v>
-      </c>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="1">
+      <c r="B2" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="18" t="s">
-        <v>76</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="F3" s="1"/>
-      <c r="G3" s="18"/>
-      <c r="H3" s="18" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="1">
+      <c r="B11" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B17" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="19" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="18" t="s">
-        <v>74</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="18"/>
-      <c r="H4" s="18" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="25">
-        <v>13</v>
-      </c>
-      <c r="B5" s="26" t="s">
+      <c r="B18" s="15">
         <v>2</v>
       </c>
-      <c r="C5" s="24" t="s">
-        <v>73</v>
-      </c>
-      <c r="D5" s="25" t="s">
-        <v>35</v>
-      </c>
-      <c r="E5" s="25" t="s">
-        <v>72</v>
-      </c>
-      <c r="F5" s="25"/>
-      <c r="G5" s="24"/>
-      <c r="H5" s="24" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="1">
-        <v>29</v>
-      </c>
-      <c r="B6" s="19" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" s="18" t="s">
-        <v>70</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="18" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="21">
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B19" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="B20" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="B24" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A25" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="22" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" s="20" t="s">
-        <v>69</v>
-      </c>
-      <c r="D7" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="20"/>
-      <c r="H7" s="20" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="1">
-        <v>53</v>
-      </c>
-      <c r="B8" s="19" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" s="18" t="s">
-        <v>67</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="18"/>
-      <c r="H8" s="18" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="1">
-        <v>32</v>
-      </c>
-      <c r="B9" s="19" t="s">
-        <v>8</v>
-      </c>
-      <c r="C9" s="18" t="s">
-        <v>66</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="18"/>
-      <c r="H9" s="18" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="1">
-        <v>52</v>
-      </c>
-      <c r="B10" s="19" t="s">
-        <v>9</v>
-      </c>
-      <c r="C10" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
-      <c r="G10" s="18"/>
-      <c r="H10" s="18" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" s="1">
-        <v>21</v>
-      </c>
-      <c r="B11" s="19" t="s">
-        <v>27</v>
-      </c>
-      <c r="C11" s="18" t="s">
-        <v>64</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-      <c r="G11" s="18"/>
-      <c r="H11" s="18" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="1">
-        <v>51</v>
-      </c>
-      <c r="B12" s="19" t="s">
-        <v>11</v>
-      </c>
-      <c r="C12" s="18" t="s">
-        <v>63</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
-      <c r="G12" s="18"/>
-      <c r="H12" s="18" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A13" s="1">
-        <v>50</v>
-      </c>
-      <c r="B13" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="C13" s="18" t="s">
-        <v>62</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="18"/>
-      <c r="H13" s="18" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A14" s="21">
-        <v>31</v>
-      </c>
-      <c r="B14" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="C14" s="20" t="s">
-        <v>61</v>
-      </c>
-      <c r="D14" s="21" t="s">
-        <v>60</v>
-      </c>
-      <c r="E14" s="20"/>
-      <c r="F14" s="20"/>
-      <c r="G14" s="20"/>
-      <c r="H14" s="20" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A15" s="1">
-        <v>15</v>
-      </c>
-      <c r="B15" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="C15" s="18" t="s">
-        <v>58</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="18"/>
-      <c r="H15" s="18" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16" s="1">
+      <c r="B25" s="15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="B26" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="19" t="s">
-        <v>15</v>
-      </c>
-      <c r="C16" s="18" t="s">
-        <v>56</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="18"/>
-      <c r="H16" s="18" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="1">
-        <v>41</v>
-      </c>
-      <c r="B17" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="C17" s="18" t="s">
-        <v>55</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="18"/>
-      <c r="H17" s="18" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A18" s="1">
+      <c r="B27" s="15">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="B18" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="C18" s="18" t="s">
-        <v>54</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="18"/>
-      <c r="H18" s="18" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A19" s="21">
-        <v>22</v>
-      </c>
-      <c r="B19" s="22" t="s">
-        <v>17</v>
-      </c>
-      <c r="C19" s="20" t="s">
-        <v>53</v>
-      </c>
-      <c r="D19" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="E19" s="21"/>
-      <c r="F19" s="21"/>
-      <c r="G19" s="20"/>
-      <c r="H19" s="20" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A20" s="1">
-        <v>33</v>
-      </c>
-      <c r="B20" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="C20" s="18" t="s">
-        <v>52</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="18"/>
-      <c r="H20" s="18" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A21" s="1">
-        <v>24</v>
-      </c>
-      <c r="B21" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="C21" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
-      <c r="G21" s="18"/>
-      <c r="H21" s="18" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A22" s="1">
-        <v>43</v>
-      </c>
-      <c r="B22" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="C22" s="18" t="s">
-        <v>48</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="18"/>
-      <c r="H22" s="18" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A23" s="1">
-        <v>11</v>
-      </c>
-      <c r="B23" s="19" t="s">
-        <v>21</v>
-      </c>
-      <c r="C23" s="18" t="s">
-        <v>47</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="E23" s="1"/>
-      <c r="F23" s="1"/>
-      <c r="G23" s="18"/>
-      <c r="H23" s="18" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A24" s="1">
-        <v>14</v>
-      </c>
-      <c r="B24" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="C24" s="18" t="s">
-        <v>46</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
-      <c r="G24" s="18"/>
-      <c r="H24" s="18" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A25" s="1">
-        <v>42</v>
-      </c>
-      <c r="B25" s="19" t="s">
-        <v>23</v>
-      </c>
-      <c r="C25" s="18" t="s">
-        <v>43</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="E25" s="1"/>
-      <c r="F25" s="1"/>
-      <c r="G25" s="18"/>
-      <c r="H25" s="23" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A26" s="1">
-        <v>35</v>
-      </c>
-      <c r="B26" s="19" t="s">
-        <v>24</v>
-      </c>
-      <c r="C26" s="18" t="s">
-        <v>40</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="E26" s="1"/>
-      <c r="F26" s="1"/>
-      <c r="G26" s="18"/>
-      <c r="H26" s="18" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A27" s="21">
-        <v>28</v>
-      </c>
-      <c r="B27" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="C27" s="20" t="s">
-        <v>39</v>
-      </c>
-      <c r="D27" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="E27" s="21" t="s">
-        <v>38</v>
-      </c>
-      <c r="F27" s="21"/>
-      <c r="G27" s="20"/>
-      <c r="H27" s="20" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A28" s="1">
-        <v>17</v>
-      </c>
-      <c r="B28" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="C28" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="E28" s="1"/>
-      <c r="F28" s="1"/>
-      <c r="G28" s="18"/>
-      <c r="H28" s="18" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A30" s="17" t="s">
-        <v>33</v>
-      </c>
-      <c r="B30" s="16"/>
-      <c r="C30" s="34" t="s">
-        <v>32</v>
-      </c>
-      <c r="D30" s="34"/>
-      <c r="E30" s="34"/>
-      <c r="F30" s="34"/>
-      <c r="G30" s="34"/>
-      <c r="H30" s="34"/>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="B31" s="15"/>
-      <c r="C31" s="34" t="s">
-        <v>31</v>
-      </c>
-      <c r="D31" s="34"/>
-      <c r="E31" s="34"/>
-      <c r="F31" s="34"/>
-      <c r="G31" s="34"/>
-      <c r="H31" s="34"/>
+      <c r="B28" s="15">
+        <v>2</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="C30:H30"/>
-    <mergeCell ref="C31:H31"/>
-  </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
ajuste difal e fcp
</commit_message>
<xml_diff>
--- a/aliquotas.xlsx
+++ b/aliquotas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Faturamento\Desktop\nfe_sistema\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E137CBC-D307-4AA1-8D3F-964228905309}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B14A8C61-B79A-4E4A-867B-FEA1B8B4A3DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9ADDC600-9F42-43BA-851C-A42DE1550295}"/>
   </bookViews>
@@ -2557,7 +2557,7 @@
         <v>12</v>
       </c>
       <c r="V22" s="12">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="W22" s="1">
         <v>7</v>

</xml_diff>